<commit_message>
actualizando cantidad de rios y paises
</commit_message>
<xml_diff>
--- a/paises.xlsx
+++ b/paises.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\martes13\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E00A8AD-88EA-48C9-B794-6AB937B5BE58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F418437E-BD21-45F2-8F03-B73AC2B75329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,9 +25,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>colombia</t>
+  </si>
+  <si>
+    <t>brasil</t>
+  </si>
+  <si>
+    <t>peru</t>
+  </si>
+  <si>
+    <t>ecuador</t>
   </si>
 </sst>
 </file>
@@ -345,7 +354,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -353,6 +362,21 @@
         <v>0</v>
       </c>
     </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>